<commit_message>
🔄 synced local 'matlabfilesuk/' with remote 'matlabMfilesUK/'
</commit_message>
<xml_diff>
--- a/matlabfilesuk/Book2ch4RegressionExt/regrStepwise.xlsx
+++ b/matlabfilesuk/Book2ch4RegressionExt/regrStepwise.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books\DataScienceWithMatlab\EserciziRiepilogoUK\Book2ch4RegressionExt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\books\DataScienceWithMatlab\matlabMfilesUK\Book2ch4RegressionExt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F176ED93-9744-4F53-A312-6AF1D401B891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E849158-A729-40CE-A54D-00B7AE579630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{B5D64D5B-A763-489F-A9D0-FEE386A4DA35}"/>
   </bookViews>
   <sheets>
-    <sheet name="Risposta11" sheetId="3" r:id="rId1"/>
+    <sheet name="data" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="aa">#REF!,#REF!</definedName>
-    <definedName name="lny">Risposta11!$L$2:$L$81</definedName>
-    <definedName name="X" localSheetId="0">Risposta11!$A$2:$J$81</definedName>
+    <definedName name="lny">data!$L$2:$L$81</definedName>
+    <definedName name="X" localSheetId="0">data!$A$2:$J$81</definedName>
     <definedName name="X">#REF!</definedName>
-    <definedName name="xstep1">Risposta11!$B$2:$J$81</definedName>
-    <definedName name="Xstep2">Risposta11!$D$87:$K$166</definedName>
-    <definedName name="xstep3">Risposta11!$D$172:$J$251</definedName>
-    <definedName name="xstep4">Risposta11!$D$258:$I$337</definedName>
-    <definedName name="xstep5">Risposta11!$D$343:$H$422</definedName>
-    <definedName name="y" localSheetId="0">Risposta11!$K$2:$K$81</definedName>
+    <definedName name="xstep1">data!$B$2:$J$81</definedName>
+    <definedName name="Xstep2">data!$D$87:$K$166</definedName>
+    <definedName name="xstep3">data!$D$172:$J$251</definedName>
+    <definedName name="xstep4">data!$D$258:$I$337</definedName>
+    <definedName name="xstep5">data!$D$343:$H$422</definedName>
+    <definedName name="y" localSheetId="0">data!$K$2:$K$81</definedName>
     <definedName name="y">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -481,7 +481,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Risposta11!$R$92</c:f>
+              <c:f>data!$R$92</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -515,7 +515,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Risposta11!$Q$93:$Q$97</c:f>
+              <c:f>data!$Q$93:$Q$97</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -539,7 +539,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Risposta11!$R$93:$R$97</c:f>
+              <c:f>data!$R$93:$R$97</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -827,7 +827,7 @@
         <xdr:cNvPr id="3104" name="Chart 29">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-0000200C0000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000200C0000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -870,7 +870,7 @@
                   <a14:compatExt spid="_x0000_s3084"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000C0C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C0C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -917,7 +917,7 @@
                   <a14:compatExt spid="_x0000_s3085"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000D0C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D0C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -964,7 +964,7 @@
                   <a14:compatExt spid="_x0000_s3086"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000E0C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E0C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1011,7 +1011,7 @@
                   <a14:compatExt spid="_x0000_s3087"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000F0C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F0C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1058,7 +1058,7 @@
                   <a14:compatExt spid="_x0000_s3088"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-0000100C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000100C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1105,7 +1105,7 @@
                   <a14:compatExt spid="_x0000_s3089"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-0000110C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000110C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1152,7 +1152,7 @@
                   <a14:compatExt spid="_x0000_s3090"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-0000120C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000120C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>

</xml_diff>